<commit_message>
Added a field in home page
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/SwagLabsTestData.xlsx
+++ b/src/test/resources/testdata/SwagLabsTestData.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bd9573b7959b23b4/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Abhi\Practice\SwagLabs\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B19A848E-C36E-4391-B077-1927017D83B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22CE3DE1-36F4-4FE2-AF2B-F84A71C7BEF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B0B95F0B-2315-45F3-9805-97334AA1DDE8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{B0B95F0B-2315-45F3-9805-97334AA1DDE8}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
+    <sheet name="Home" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
   <si>
     <t>username</t>
   </si>
@@ -49,6 +50,18 @@
   </si>
   <si>
     <t>problem_user</t>
+  </si>
+  <si>
+    <t>ItemToAdd</t>
+  </si>
+  <si>
+    <t>Sauce Labs Backpack</t>
+  </si>
+  <si>
+    <t>Sauce Labs Bike Light</t>
+  </si>
+  <si>
+    <t>Sauce Labs Onesie</t>
   </si>
 </sst>
 </file>
@@ -437,4 +450,34 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57B5FFEE-6253-47EC-8284-3B526E194786}">
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>